<commit_message>
Part D: focus on B4 only
Drop the B6 analysis from Part D and the register; keep the 6-piece only
where it bids in B4's auctions (a cause of B4's low top-of-search share).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FvXHKtbYmE3ru99HYV2muV
</commit_message>
<xml_diff>
--- a/docs/DBS4_Corrections_by_Situation_20260921-dbcd48b8.xlsx
+++ b/docs/DBS4_Corrections_by_Situation_20260921-dbcd48b8.xlsx
@@ -10,8 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ranking campaigns" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Other campaign types" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B4 keyword diagnosis" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B6 keyword diagnosis" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Syntax groups" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Syntax groups" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ranking campaigns'!$A$1:$Q$214</definedName>
@@ -18754,2526 +18753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V41"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="21" max="21"/>
-    <col width="80" customWidth="1" min="22" max="22"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Keyword</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Syntax</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Plan clicks/wk</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Weekly SV</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Clicks 30d</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>TOS clicks 30d</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>TOS clicks/day pre-deal</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>TOS clicks/day deal</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>TOS share</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>TOS CTR</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>CTR bar</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>TOS CVR</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>CVR bar</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>TOS impr. share</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Eff. TOS bid</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Organic</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Sponsored</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Rank 24 Jun</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Rank 14 Sep</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Rank 22 Sep</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Verdict</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Recommendation</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>bamboo sheets</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Bamboo</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>47605</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1036</v>
-      </c>
-      <c r="F2" t="n">
-        <v>382</v>
-      </c>
-      <c r="G2" t="n">
-        <v>15.2</v>
-      </c>
-      <c r="H2" t="n">
-        <v>6</v>
-      </c>
-      <c r="I2" t="n">
-        <v>37</v>
-      </c>
-      <c r="J2" t="n">
-        <v>3.01</v>
-      </c>
-      <c r="K2" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="L2" t="n">
-        <v>18.84</v>
-      </c>
-      <c r="M2" t="n">
-        <v>8.31</v>
-      </c>
-      <c r="N2" t="n">
-        <v>2.06</v>
-      </c>
-      <c r="O2" t="n">
-        <v>6.1</v>
-      </c>
-      <c r="P2" t="n">
-        <v>36</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>19</v>
-      </c>
-      <c r="R2" t="n">
-        <v>23</v>
-      </c>
-      <c r="S2" t="n">
-        <v>25</v>
-      </c>
-      <c r="T2" t="n">
-        <v>35</v>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>viscose bamboo sheets</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Bamboo</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>642</v>
-      </c>
-      <c r="E3" t="n">
-        <v>169</v>
-      </c>
-      <c r="F3" t="n">
-        <v>57</v>
-      </c>
-      <c r="G3" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="H3" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="I3" t="n">
-        <v>34</v>
-      </c>
-      <c r="J3" t="n">
-        <v>4.65</v>
-      </c>
-      <c r="K3" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="L3" t="n">
-        <v>23.4</v>
-      </c>
-      <c r="M3" t="n">
-        <v>8.31</v>
-      </c>
-      <c r="N3" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="O3" t="n">
-        <v>5.95</v>
-      </c>
-      <c r="P3" t="n">
-        <v>12</v>
-      </c>
-      <c r="R3" t="n">
-        <v>16</v>
-      </c>
-      <c r="S3" t="n">
-        <v>13</v>
-      </c>
-      <c r="T3" t="n">
-        <v>13</v>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>king size bamboo sheets set</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Bamboo|King</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>1367</v>
-      </c>
-      <c r="E4" t="n">
-        <v>128</v>
-      </c>
-      <c r="F4" t="n">
-        <v>47</v>
-      </c>
-      <c r="G4" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I4" t="n">
-        <v>37</v>
-      </c>
-      <c r="J4" t="n">
-        <v>7.19</v>
-      </c>
-      <c r="K4" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="L4" t="n">
-        <v>18.66</v>
-      </c>
-      <c r="M4" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="N4" t="n">
-        <v>7.13</v>
-      </c>
-      <c r="O4" t="n">
-        <v>7.33</v>
-      </c>
-      <c r="P4" t="n">
-        <v>29</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>4</v>
-      </c>
-      <c r="R4" t="n">
-        <v>9</v>
-      </c>
-      <c r="S4" t="n">
-        <v>29</v>
-      </c>
-      <c r="T4" t="n">
-        <v>36</v>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>bamboo sheets queen size</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Bamboo|Queen</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>10342</v>
-      </c>
-      <c r="E5" t="n">
-        <v>166</v>
-      </c>
-      <c r="F5" t="n">
-        <v>38</v>
-      </c>
-      <c r="G5" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="I5" t="n">
-        <v>23</v>
-      </c>
-      <c r="J5" t="n">
-        <v>5.92</v>
-      </c>
-      <c r="K5" t="n">
-        <v>1.81</v>
-      </c>
-      <c r="L5" t="n">
-        <v>32.84</v>
-      </c>
-      <c r="M5" t="n">
-        <v>13.32</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="O5" t="n">
-        <v>4.56</v>
-      </c>
-      <c r="P5" t="n">
-        <v>36</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>4</v>
-      </c>
-      <c r="R5" t="n">
-        <v>28</v>
-      </c>
-      <c r="S5" t="n">
-        <v>32</v>
-      </c>
-      <c r="T5" t="n">
-        <v>32</v>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>bamboo bed sheets</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Bamboo</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>1564</v>
-      </c>
-      <c r="E6" t="n">
-        <v>44</v>
-      </c>
-      <c r="F6" t="n">
-        <v>35</v>
-      </c>
-      <c r="G6" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="I6" t="n">
-        <v>78</v>
-      </c>
-      <c r="J6" t="n">
-        <v>3.69</v>
-      </c>
-      <c r="K6" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="L6" t="n">
-        <v>16.88</v>
-      </c>
-      <c r="M6" t="n">
-        <v>8.31</v>
-      </c>
-      <c r="N6" t="n">
-        <v>1.76</v>
-      </c>
-      <c r="O6" t="n">
-        <v>6.58</v>
-      </c>
-      <c r="P6" t="n">
-        <v>40</v>
-      </c>
-      <c r="R6" t="n">
-        <v>31</v>
-      </c>
-      <c r="S6" t="n">
-        <v>31</v>
-      </c>
-      <c r="T6" t="n">
-        <v>27</v>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>bamboo sheets with corner straps</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Bamboo</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>115</v>
-      </c>
-      <c r="E7" t="n">
-        <v>75</v>
-      </c>
-      <c r="F7" t="n">
-        <v>29</v>
-      </c>
-      <c r="G7" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="I7" t="n">
-        <v>39</v>
-      </c>
-      <c r="J7" t="n">
-        <v>6.72</v>
-      </c>
-      <c r="K7" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="L7" t="n">
-        <v>21.67</v>
-      </c>
-      <c r="M7" t="n">
-        <v>8.31</v>
-      </c>
-      <c r="N7" t="n">
-        <v>14.21</v>
-      </c>
-      <c r="O7" t="n">
-        <v>5.62</v>
-      </c>
-      <c r="P7" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>1</v>
-      </c>
-      <c r="R7" t="n">
-        <v>23</v>
-      </c>
-      <c r="S7" t="n">
-        <v>13</v>
-      </c>
-      <c r="T7" t="n">
-        <v>14</v>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>ON TRACK</t>
-        </is>
-      </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>Meets the CTR/CVR bars and wins TOS: scale while rank moves; if rank stalls, the gap is volume vs rivals — raise by the rank-gap step.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>queen sheet set bamboo</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Bamboo|Queen</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>366</v>
-      </c>
-      <c r="E8" t="n">
-        <v>97</v>
-      </c>
-      <c r="F8" t="n">
-        <v>2</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>2</v>
-      </c>
-      <c r="K8" t="n">
-        <v>1.81</v>
-      </c>
-      <c r="M8" t="n">
-        <v>13.32</v>
-      </c>
-      <c r="P8" t="n">
-        <v>40</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>2</v>
-      </c>
-      <c r="R8" t="n">
-        <v>18</v>
-      </c>
-      <c r="S8" t="n">
-        <v>35</v>
-      </c>
-      <c r="T8" t="n">
-        <v>44</v>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>Eligibility first: confirm the exact campaign is enabled and its TOS price clears the group market limit; then push +25% on TOS and read in 3 days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>bamboo king sheets</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Bamboo|King</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>1148</v>
-      </c>
-      <c r="E9" t="n">
-        <v>33</v>
-      </c>
-      <c r="F9" t="n">
-        <v>30</v>
-      </c>
-      <c r="G9" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="I9" t="n">
-        <v>90</v>
-      </c>
-      <c r="J9" t="n">
-        <v>5.26</v>
-      </c>
-      <c r="K9" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="M9" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="N9" t="n">
-        <v>6.66</v>
-      </c>
-      <c r="O9" t="n">
-        <v>7.07</v>
-      </c>
-      <c r="P9" t="n">
-        <v>23</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>17</v>
-      </c>
-      <c r="R9" t="n">
-        <v>16</v>
-      </c>
-      <c r="S9" t="n">
-        <v>15</v>
-      </c>
-      <c r="T9" t="n">
-        <v>18</v>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>bamboo sheets full</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Bamboo|Full</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>1588</v>
-      </c>
-      <c r="E10" t="n">
-        <v>51</v>
-      </c>
-      <c r="F10" t="n">
-        <v>35</v>
-      </c>
-      <c r="G10" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="H10" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="I10" t="n">
-        <v>69</v>
-      </c>
-      <c r="J10" t="n">
-        <v>4.07</v>
-      </c>
-      <c r="K10" t="n">
-        <v>2.06</v>
-      </c>
-      <c r="M10" t="n">
-        <v>12.18</v>
-      </c>
-      <c r="N10" t="n">
-        <v>1.18</v>
-      </c>
-      <c r="O10" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="P10" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>7</v>
-      </c>
-      <c r="R10" t="n">
-        <v>58</v>
-      </c>
-      <c r="S10" t="n">
-        <v>13</v>
-      </c>
-      <c r="T10" t="n">
-        <v>11</v>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>king bamboo sheets</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Bamboo|King</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>1355</v>
-      </c>
-      <c r="E11" t="n">
-        <v>59</v>
-      </c>
-      <c r="F11" t="n">
-        <v>12</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" t="n">
-        <v>21</v>
-      </c>
-      <c r="J11" t="n">
-        <v>1.94</v>
-      </c>
-      <c r="K11" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="M11" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="P11" t="n">
-        <v>32</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>9</v>
-      </c>
-      <c r="R11" t="n">
-        <v>23</v>
-      </c>
-      <c r="S11" t="n">
-        <v>31</v>
-      </c>
-      <c r="T11" t="n">
-        <v>40</v>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>BOTH — short of traffic and under target</t>
-        </is>
-      </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>Fix the offer first, then buy traffic: a small TOS probe (+10%) only while the CTR/CVR fix is made.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>bamboo sheets king size</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Bamboo|King</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>6945</v>
-      </c>
-      <c r="E12" t="n">
-        <v>54</v>
-      </c>
-      <c r="F12" t="n">
-        <v>17</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="I12" t="n">
-        <v>32</v>
-      </c>
-      <c r="J12" t="n">
-        <v>4.89</v>
-      </c>
-      <c r="K12" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="M12" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="N12" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="O12" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="P12" t="n">
-        <v>37</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>19</v>
-      </c>
-      <c r="R12" t="n">
-        <v>15</v>
-      </c>
-      <c r="S12" t="n">
-        <v>36</v>
-      </c>
-      <c r="T12" t="n">
-        <v>38</v>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>red bamboo sheets</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>53</v>
-      </c>
-      <c r="F13" t="n">
-        <v>25</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="I13" t="n">
-        <v>45</v>
-      </c>
-      <c r="J13" t="n">
-        <v>8.960000000000001</v>
-      </c>
-      <c r="L13" t="n">
-        <v>16.57</v>
-      </c>
-      <c r="N13" t="n">
-        <v>26.58</v>
-      </c>
-      <c r="O13" t="n">
-        <v>4.78</v>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>black bamboo sheets</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Bamboo</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>463</v>
-      </c>
-      <c r="E14" t="n">
-        <v>30</v>
-      </c>
-      <c r="F14" t="n">
-        <v>19</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="I14" t="n">
-        <v>62</v>
-      </c>
-      <c r="J14" t="n">
-        <v>4.19</v>
-      </c>
-      <c r="K14" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="M14" t="n">
-        <v>8.31</v>
-      </c>
-      <c r="N14" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="O14" t="n">
-        <v>4.82</v>
-      </c>
-      <c r="P14" t="n">
-        <v>13</v>
-      </c>
-      <c r="R14" t="n">
-        <v>18</v>
-      </c>
-      <c r="S14" t="n">
-        <v>21</v>
-      </c>
-      <c r="T14" t="n">
-        <v>17</v>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>bamboo cooling sheets</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Bamboo|Cooling</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>3233</v>
-      </c>
-      <c r="E15" t="n">
-        <v>44</v>
-      </c>
-      <c r="F15" t="n">
-        <v>3</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="I15" t="n">
-        <v>7</v>
-      </c>
-      <c r="K15" t="n">
-        <v>2.07</v>
-      </c>
-      <c r="L15" t="n">
-        <v>17.26</v>
-      </c>
-      <c r="M15" t="n">
-        <v>7.71</v>
-      </c>
-      <c r="N15" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="O15" t="n">
-        <v>3.16</v>
-      </c>
-      <c r="P15" t="n">
-        <v>36</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>17</v>
-      </c>
-      <c r="R15" t="n">
-        <v>30</v>
-      </c>
-      <c r="S15" t="n">
-        <v>35</v>
-      </c>
-      <c r="T15" t="n">
-        <v>27</v>
-      </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>Eligibility first: confirm the exact campaign is enabled and its TOS price clears the group market limit; then push +25% on TOS and read in 3 days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>bamboo sheet set</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Bamboo</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>545</v>
-      </c>
-      <c r="E16" t="n">
-        <v>31</v>
-      </c>
-      <c r="F16" t="n">
-        <v>16</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" t="n">
-        <v>51</v>
-      </c>
-      <c r="J16" t="n">
-        <v>4.26</v>
-      </c>
-      <c r="K16" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="M16" t="n">
-        <v>8.31</v>
-      </c>
-      <c r="N16" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="O16" t="n">
-        <v>4.47</v>
-      </c>
-      <c r="P16" t="n">
-        <v>58</v>
-      </c>
-      <c r="R16" t="n">
-        <v>22</v>
-      </c>
-      <c r="S16" t="n">
-        <v>48</v>
-      </c>
-      <c r="T16" t="n">
-        <v>38</v>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>burgundy sheets queen</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>352</v>
-      </c>
-      <c r="E17" t="n">
-        <v>27</v>
-      </c>
-      <c r="F17" t="n">
-        <v>9</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="I17" t="n">
-        <v>33</v>
-      </c>
-      <c r="P17" t="n">
-        <v>31</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>5</v>
-      </c>
-      <c r="R17" t="n">
-        <v>47</v>
-      </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>Eligibility first: confirm the exact campaign is enabled and its TOS price clears the group market limit; then push +25% on TOS and read in 3 days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>full bamboo sheets</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Bamboo|Full</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>200</v>
-      </c>
-      <c r="E18" t="n">
-        <v>22</v>
-      </c>
-      <c r="F18" t="n">
-        <v>10</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="I18" t="n">
-        <v>45</v>
-      </c>
-      <c r="J18" t="n">
-        <v>8.039999999999999</v>
-      </c>
-      <c r="K18" t="n">
-        <v>2.06</v>
-      </c>
-      <c r="M18" t="n">
-        <v>12.18</v>
-      </c>
-      <c r="N18" t="n">
-        <v>5.62</v>
-      </c>
-      <c r="O18" t="n">
-        <v>6.45</v>
-      </c>
-      <c r="P18" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>1</v>
-      </c>
-      <c r="R18" t="n">
-        <v>15</v>
-      </c>
-      <c r="S18" t="n">
-        <v>12</v>
-      </c>
-      <c r="T18" t="n">
-        <v>13</v>
-      </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>bamboo twin sheets</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Bamboo|Twin</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>417</v>
-      </c>
-      <c r="E19" t="n">
-        <v>20</v>
-      </c>
-      <c r="F19" t="n">
-        <v>7</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" t="n">
-        <v>35</v>
-      </c>
-      <c r="J19" t="n">
-        <v>3.92</v>
-      </c>
-      <c r="K19" t="n">
-        <v>2.07</v>
-      </c>
-      <c r="M19" t="n">
-        <v>10.95</v>
-      </c>
-      <c r="P19" t="n">
-        <v>28</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>18</v>
-      </c>
-      <c r="R19" t="n">
-        <v>13</v>
-      </c>
-      <c r="S19" t="n">
-        <v>28</v>
-      </c>
-      <c r="T19" t="n">
-        <v>25</v>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>bamboo full size bed sheets</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Bamboo|Full</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>197</v>
-      </c>
-      <c r="E20" t="n">
-        <v>14</v>
-      </c>
-      <c r="F20" t="n">
-        <v>13</v>
-      </c>
-      <c r="G20" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="I20" t="n">
-        <v>89</v>
-      </c>
-      <c r="J20" t="n">
-        <v>10.83</v>
-      </c>
-      <c r="K20" t="n">
-        <v>2.06</v>
-      </c>
-      <c r="L20" t="n">
-        <v>40.5</v>
-      </c>
-      <c r="M20" t="n">
-        <v>12.18</v>
-      </c>
-      <c r="P20" t="n">
-        <v>28</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>20</v>
-      </c>
-      <c r="R20" t="n">
-        <v>36</v>
-      </c>
-      <c r="S20" t="n">
-        <v>25</v>
-      </c>
-      <c r="T20" t="n">
-        <v>26</v>
-      </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>bamboo sheets queen</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Bamboo|Queen</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>858</v>
-      </c>
-      <c r="E21" t="n">
-        <v>37</v>
-      </c>
-      <c r="F21" t="n">
-        <v>7</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" t="n">
-        <v>20</v>
-      </c>
-      <c r="K21" t="n">
-        <v>1.81</v>
-      </c>
-      <c r="M21" t="n">
-        <v>13.32</v>
-      </c>
-      <c r="N21" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="O21" t="n">
-        <v>3.52</v>
-      </c>
-      <c r="P21" t="n">
-        <v>63</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>8</v>
-      </c>
-      <c r="R21" t="n">
-        <v>18</v>
-      </c>
-      <c r="S21" t="n">
-        <v>39</v>
-      </c>
-      <c r="T21" t="n">
-        <v>55</v>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>Eligibility first: confirm the exact campaign is enabled and its TOS price clears the group market limit; then push +25% on TOS and read in 3 days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>sheets queen size bed set</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>23315</v>
-      </c>
-      <c r="E22" t="n">
-        <v>41</v>
-      </c>
-      <c r="F22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I22" t="n">
-        <v>3</v>
-      </c>
-      <c r="L22" t="n">
-        <v>18.52</v>
-      </c>
-      <c r="P22" t="n">
-        <v>71</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>17</v>
-      </c>
-      <c r="R22" t="n">
-        <v>48</v>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>Eligibility first: confirm the exact campaign is enabled and its TOS price clears the group market limit; then push +25% on TOS and read in 3 days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>cooling bed sheets</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Cooling</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>5185</v>
-      </c>
-      <c r="E23" t="n">
-        <v>20</v>
-      </c>
-      <c r="F23" t="n">
-        <v>12</v>
-      </c>
-      <c r="G23" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="I23" t="n">
-        <v>59</v>
-      </c>
-      <c r="K23" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="M23" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="P23" t="n">
-        <v>34</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>22</v>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>Eligibility first: confirm the exact campaign is enabled and its TOS price clears the group market limit; then push +25% on TOS and read in 3 days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>twin sheets bamboo</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Bamboo|Twin</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>203</v>
-      </c>
-      <c r="E24" t="n">
-        <v>21</v>
-      </c>
-      <c r="F24" t="n">
-        <v>8</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" t="n">
-        <v>38</v>
-      </c>
-      <c r="K24" t="n">
-        <v>2.07</v>
-      </c>
-      <c r="M24" t="n">
-        <v>10.95</v>
-      </c>
-      <c r="P24" t="n">
-        <v>34</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>1</v>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>Eligibility first: confirm the exact campaign is enabled and its TOS price clears the group market limit; then push +25% on TOS and read in 3 days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>bamboo sheets pink</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>29</v>
-      </c>
-      <c r="F25" t="n">
-        <v>3</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" t="n">
-        <v>11</v>
-      </c>
-      <c r="J25" t="n">
-        <v>2.97</v>
-      </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>full size bamboo sheets</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Bamboo|Full</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>460</v>
-      </c>
-      <c r="E26" t="n">
-        <v>18</v>
-      </c>
-      <c r="F26" t="n">
-        <v>8</v>
-      </c>
-      <c r="G26" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" t="n">
-        <v>46</v>
-      </c>
-      <c r="J26" t="n">
-        <v>6.58</v>
-      </c>
-      <c r="K26" t="n">
-        <v>2.06</v>
-      </c>
-      <c r="M26" t="n">
-        <v>12.18</v>
-      </c>
-      <c r="N26" t="n">
-        <v>3.35</v>
-      </c>
-      <c r="O26" t="n">
-        <v>6.49</v>
-      </c>
-      <c r="P26" t="n">
-        <v>39</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>15</v>
-      </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>bamboo viscose sheets queen size</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Bamboo|Queen</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>124</v>
-      </c>
-      <c r="E27" t="n">
-        <v>15</v>
-      </c>
-      <c r="F27" t="n">
-        <v>9</v>
-      </c>
-      <c r="G27" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="H27" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" t="n">
-        <v>59</v>
-      </c>
-      <c r="J27" t="n">
-        <v>3.98</v>
-      </c>
-      <c r="K27" t="n">
-        <v>1.81</v>
-      </c>
-      <c r="M27" t="n">
-        <v>13.32</v>
-      </c>
-      <c r="P27" t="n">
-        <v>23</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>1</v>
-      </c>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>bamboo sheets twin</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Bamboo|Twin</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>714</v>
-      </c>
-      <c r="E28" t="n">
-        <v>26</v>
-      </c>
-      <c r="F28" t="n">
-        <v>2</v>
-      </c>
-      <c r="G28" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="H28" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" t="n">
-        <v>9</v>
-      </c>
-      <c r="K28" t="n">
-        <v>2.07</v>
-      </c>
-      <c r="M28" t="n">
-        <v>10.95</v>
-      </c>
-      <c r="P28" t="n">
-        <v>24</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>24</v>
-      </c>
-      <c r="U28" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>Eligibility first: confirm the exact campaign is enabled and its TOS price clears the group market limit; then push +25% on TOS and read in 3 days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>100% bamboo sheets king size</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Bamboo|King</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>260</v>
-      </c>
-      <c r="E29" t="n">
-        <v>18</v>
-      </c>
-      <c r="F29" t="n">
-        <v>4</v>
-      </c>
-      <c r="G29" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="H29" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="I29" t="n">
-        <v>24</v>
-      </c>
-      <c r="J29" t="n">
-        <v>4.26</v>
-      </c>
-      <c r="K29" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="M29" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="P29" t="n">
-        <v>39</v>
-      </c>
-      <c r="Q29" t="n">
-        <v>15</v>
-      </c>
-      <c r="U29" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V29" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>king bamboo sheets deep pocket</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Bamboo|King</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>355</v>
-      </c>
-      <c r="E30" t="n">
-        <v>13</v>
-      </c>
-      <c r="F30" t="n">
-        <v>6</v>
-      </c>
-      <c r="G30" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" t="n">
-        <v>43</v>
-      </c>
-      <c r="J30" t="n">
-        <v>4.69</v>
-      </c>
-      <c r="K30" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="M30" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="P30" t="n">
-        <v>34</v>
-      </c>
-      <c r="Q30" t="n">
-        <v>1</v>
-      </c>
-      <c r="U30" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V30" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>bamboo sheet sets</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Bamboo</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>121</v>
-      </c>
-      <c r="E31" t="n">
-        <v>10</v>
-      </c>
-      <c r="F31" t="n">
-        <v>6</v>
-      </c>
-      <c r="G31" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" t="n">
-        <v>56</v>
-      </c>
-      <c r="K31" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="M31" t="n">
-        <v>8.31</v>
-      </c>
-      <c r="N31" t="n">
-        <v>4.02</v>
-      </c>
-      <c r="O31" t="n">
-        <v>4.47</v>
-      </c>
-      <c r="P31" t="n">
-        <v>36</v>
-      </c>
-      <c r="Q31" t="n">
-        <v>12</v>
-      </c>
-      <c r="U31" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-      <c r="V31" t="inlineStr">
-        <is>
-          <t>Eligibility first: confirm the exact campaign is enabled and its TOS price clears the group market limit; then push +25% on TOS and read in 3 days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>queen bamboo sheet set</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Bamboo|Queen</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>1397</v>
-      </c>
-      <c r="E32" t="n">
-        <v>15</v>
-      </c>
-      <c r="F32" t="n">
-        <v>7</v>
-      </c>
-      <c r="G32" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H32" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I32" t="n">
-        <v>48</v>
-      </c>
-      <c r="K32" t="n">
-        <v>1.81</v>
-      </c>
-      <c r="M32" t="n">
-        <v>13.32</v>
-      </c>
-      <c r="N32" t="n">
-        <v>1.11</v>
-      </c>
-      <c r="O32" t="n">
-        <v>6.07</v>
-      </c>
-      <c r="P32" t="n">
-        <v>21</v>
-      </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-      <c r="V32" t="inlineStr">
-        <is>
-          <t>Eligibility first: confirm the exact campaign is enabled and its TOS price clears the group market limit; then push +25% on TOS and read in 3 days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>queen size sheets bamboo</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Bamboo|Queen</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>107</v>
-      </c>
-      <c r="E33" t="n">
-        <v>7</v>
-      </c>
-      <c r="F33" t="n">
-        <v>7</v>
-      </c>
-      <c r="G33" t="n">
-        <v>0</v>
-      </c>
-      <c r="H33" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="I33" t="n">
-        <v>100</v>
-      </c>
-      <c r="K33" t="n">
-        <v>1.81</v>
-      </c>
-      <c r="M33" t="n">
-        <v>13.32</v>
-      </c>
-      <c r="P33" t="n">
-        <v>40</v>
-      </c>
-      <c r="Q33" t="n">
-        <v>3</v>
-      </c>
-      <c r="U33" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-      <c r="V33" t="inlineStr">
-        <is>
-          <t>Eligibility first: confirm the exact campaign is enabled and its TOS price clears the group market limit; then push +25% on TOS and read in 3 days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>king bed bamboo sheets</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Bamboo|King</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>319</v>
-      </c>
-      <c r="E34" t="n">
-        <v>11</v>
-      </c>
-      <c r="F34" t="n">
-        <v>5</v>
-      </c>
-      <c r="G34" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H34" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I34" t="n">
-        <v>49</v>
-      </c>
-      <c r="J34" t="n">
-        <v>3.24</v>
-      </c>
-      <c r="K34" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="M34" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="P34" t="n">
-        <v>22</v>
-      </c>
-      <c r="Q34" t="n">
-        <v>27</v>
-      </c>
-      <c r="U34" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V34" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>cooling bed sheets king</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Cooling|King</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>492</v>
-      </c>
-      <c r="E35" t="n">
-        <v>8</v>
-      </c>
-      <c r="F35" t="n">
-        <v>7</v>
-      </c>
-      <c r="G35" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H35" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="I35" t="n">
-        <v>90</v>
-      </c>
-      <c r="J35" t="n">
-        <v>6.71</v>
-      </c>
-      <c r="K35" t="n">
-        <v>2.16</v>
-      </c>
-      <c r="M35" t="n">
-        <v>10.53</v>
-      </c>
-      <c r="P35" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q35" t="n">
-        <v>11</v>
-      </c>
-      <c r="U35" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V35" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>bamboo sheets california king</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Bamboo|California King</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>420</v>
-      </c>
-      <c r="E36" t="n">
-        <v>17</v>
-      </c>
-      <c r="F36" t="n">
-        <v>1</v>
-      </c>
-      <c r="G36" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" t="n">
-        <v>0</v>
-      </c>
-      <c r="I36" t="n">
-        <v>5</v>
-      </c>
-      <c r="K36" t="n">
-        <v>2.07</v>
-      </c>
-      <c r="M36" t="n">
-        <v>8.85</v>
-      </c>
-      <c r="N36" t="n">
-        <v>2.14</v>
-      </c>
-      <c r="O36" t="n">
-        <v>2.84</v>
-      </c>
-      <c r="P36" t="n">
-        <v>29</v>
-      </c>
-      <c r="Q36" t="n">
-        <v>6</v>
-      </c>
-      <c r="U36" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-      <c r="V36" t="inlineStr">
-        <is>
-          <t>Eligibility first: confirm the exact campaign is enabled and its TOS price clears the group market limit; then push +25% on TOS and read in 3 days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>queen sheets set bamboo</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>18</v>
-      </c>
-      <c r="F37" t="n">
-        <v>0</v>
-      </c>
-      <c r="G37" t="n">
-        <v>0</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" t="n">
-        <v>2</v>
-      </c>
-      <c r="N37" t="n">
-        <v>2.72</v>
-      </c>
-      <c r="O37" t="n">
-        <v>4.72</v>
-      </c>
-      <c r="U37" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-      <c r="V37" t="inlineStr">
-        <is>
-          <t>Eligibility first: confirm the exact campaign is enabled and its TOS price clears the group market limit; then push +25% on TOS and read in 3 days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>bamboo sheets king</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Bamboo|King</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
-        <v>2680</v>
-      </c>
-      <c r="E38" t="n">
-        <v>11</v>
-      </c>
-      <c r="F38" t="n">
-        <v>8</v>
-      </c>
-      <c r="G38" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="H38" t="n">
-        <v>0</v>
-      </c>
-      <c r="I38" t="n">
-        <v>74</v>
-      </c>
-      <c r="K38" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="M38" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="N38" t="n">
-        <v>1.11</v>
-      </c>
-      <c r="O38" t="n">
-        <v>4.75</v>
-      </c>
-      <c r="P38" t="n">
-        <v>28</v>
-      </c>
-      <c r="Q38" t="n">
-        <v>19</v>
-      </c>
-      <c r="U38" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-      <c r="V38" t="inlineStr">
-        <is>
-          <t>Eligibility first: confirm the exact campaign is enabled and its TOS price clears the group market limit; then push +25% on TOS and read in 3 days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>bamboo king size sheets</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Bamboo|King</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>132</v>
-      </c>
-      <c r="E39" t="n">
-        <v>8</v>
-      </c>
-      <c r="F39" t="n">
-        <v>5</v>
-      </c>
-      <c r="G39" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="H39" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="I39" t="n">
-        <v>67</v>
-      </c>
-      <c r="K39" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="M39" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="P39" t="n">
-        <v>38</v>
-      </c>
-      <c r="Q39" t="n">
-        <v>17</v>
-      </c>
-      <c r="U39" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-      <c r="V39" t="inlineStr">
-        <is>
-          <t>Eligibility first: confirm the exact campaign is enabled and its TOS price clears the group market limit; then push +25% on TOS and read in 3 days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>extra deep 20-24 inch pocket king size bamboo sheets</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Bamboo|King</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>175</v>
-      </c>
-      <c r="E40" t="n">
-        <v>8</v>
-      </c>
-      <c r="F40" t="n">
-        <v>7</v>
-      </c>
-      <c r="G40" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H40" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="I40" t="n">
-        <v>91</v>
-      </c>
-      <c r="K40" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="L40" t="n">
-        <v>0</v>
-      </c>
-      <c r="M40" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="P40" t="n">
-        <v>93</v>
-      </c>
-      <c r="Q40" t="n">
-        <v>2</v>
-      </c>
-      <c r="U40" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-      <c r="V40" t="inlineStr">
-        <is>
-          <t>Eligibility first: confirm the exact campaign is enabled and its TOS price clears the group market limit; then push +25% on TOS and read in 3 days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>king sheets bamboo</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Bamboo|King</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
-        <v>766</v>
-      </c>
-      <c r="E41" t="n">
-        <v>10</v>
-      </c>
-      <c r="F41" t="n">
-        <v>5</v>
-      </c>
-      <c r="G41" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H41" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I41" t="n">
-        <v>46</v>
-      </c>
-      <c r="J41" t="n">
-        <v>2.44</v>
-      </c>
-      <c r="K41" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="M41" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="N41" t="n">
-        <v>1.27</v>
-      </c>
-      <c r="O41" t="n">
-        <v>7.93</v>
-      </c>
-      <c r="P41" t="n">
-        <v>26</v>
-      </c>
-      <c r="Q41" t="n">
-        <v>25</v>
-      </c>
-      <c r="U41" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-      <c r="V41" t="inlineStr">
-        <is>
-          <t>Buy the traffic: it converts at top of search. Raise the TOS modifier by the rank-gap step, lift budget if it caps, and hold base so PDP does not grow.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Q38"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="2" max="2"/>
@@ -22356,969 +19836,6 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>B6</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Bamboo</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>12098.02</v>
-      </c>
-      <c r="D21" t="n">
-        <v>3843</v>
-      </c>
-      <c r="E21" t="n">
-        <v>565</v>
-      </c>
-      <c r="F21" t="n">
-        <v>40</v>
-      </c>
-      <c r="G21" t="n">
-        <v>3.47</v>
-      </c>
-      <c r="H21" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="I21" t="n">
-        <v>17.57</v>
-      </c>
-      <c r="J21" t="n">
-        <v>8.31</v>
-      </c>
-      <c r="K21" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L21" t="n">
-        <v>5.49</v>
-      </c>
-      <c r="M21" t="n">
-        <v>21</v>
-      </c>
-      <c r="N21" t="n">
-        <v>25</v>
-      </c>
-      <c r="O21" t="n">
-        <v>30</v>
-      </c>
-      <c r="P21" t="n">
-        <v>31</v>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>B6</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Bamboo|King</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>1749.089999999999</v>
-      </c>
-      <c r="D22" t="n">
-        <v>427</v>
-      </c>
-      <c r="E22" t="n">
-        <v>185</v>
-      </c>
-      <c r="F22" t="n">
-        <v>45</v>
-      </c>
-      <c r="G22" t="n">
-        <v>5.99</v>
-      </c>
-      <c r="H22" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="I22" t="n">
-        <v>4.74</v>
-      </c>
-      <c r="J22" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="K22" t="n">
-        <v>4.91</v>
-      </c>
-      <c r="L22" t="n">
-        <v>6.08</v>
-      </c>
-      <c r="M22" t="n">
-        <v>20</v>
-      </c>
-      <c r="N22" t="n">
-        <v>21</v>
-      </c>
-      <c r="O22" t="n">
-        <v>29</v>
-      </c>
-      <c r="P22" t="n">
-        <v>35</v>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>BOTH — short of traffic and under target</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>B6</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Bamboo|Queen</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>1320.28</v>
-      </c>
-      <c r="D23" t="n">
-        <v>470</v>
-      </c>
-      <c r="E23" t="n">
-        <v>123</v>
-      </c>
-      <c r="F23" t="n">
-        <v>28</v>
-      </c>
-      <c r="G23" t="n">
-        <v>7.78</v>
-      </c>
-      <c r="H23" t="n">
-        <v>1.81</v>
-      </c>
-      <c r="I23" t="n">
-        <v>10.24</v>
-      </c>
-      <c r="J23" t="n">
-        <v>13.32</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="L23" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="M23" t="n">
-        <v>18</v>
-      </c>
-      <c r="N23" t="n">
-        <v>29</v>
-      </c>
-      <c r="O23" t="n">
-        <v>35</v>
-      </c>
-      <c r="P23" t="n">
-        <v>41</v>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>BOTH — short of traffic and under target</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>B6</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Cooling</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>930.33</v>
-      </c>
-      <c r="D24" t="n">
-        <v>337</v>
-      </c>
-      <c r="E24" t="n">
-        <v>16</v>
-      </c>
-      <c r="F24" t="n">
-        <v>49</v>
-      </c>
-      <c r="G24" t="n">
-        <v>11.01</v>
-      </c>
-      <c r="H24" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="I24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="L24" t="n">
-        <v>4.37</v>
-      </c>
-      <c r="M24" t="n">
-        <v>52</v>
-      </c>
-      <c r="N24" t="n">
-        <v>52</v>
-      </c>
-      <c r="O24" t="n">
-        <v>55</v>
-      </c>
-      <c r="P24" t="n">
-        <v>60</v>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>BOTH — short of traffic and under target</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>B6</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Bamboo|Full</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>615.8000000000002</v>
-      </c>
-      <c r="D25" t="n">
-        <v>147</v>
-      </c>
-      <c r="E25" t="n">
-        <v>91</v>
-      </c>
-      <c r="F25" t="n">
-        <v>64</v>
-      </c>
-      <c r="G25" t="n">
-        <v>6.71</v>
-      </c>
-      <c r="H25" t="n">
-        <v>2.06</v>
-      </c>
-      <c r="I25" t="n">
-        <v>5.95</v>
-      </c>
-      <c r="J25" t="n">
-        <v>12.18</v>
-      </c>
-      <c r="K25" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="L25" t="n">
-        <v>5</v>
-      </c>
-      <c r="M25" t="n">
-        <v>27</v>
-      </c>
-      <c r="N25" t="n">
-        <v>17</v>
-      </c>
-      <c r="O25" t="n">
-        <v>20</v>
-      </c>
-      <c r="P25" t="n">
-        <v>23</v>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>BOTH — short of traffic and under target</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>B6</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Size: Queen</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>575.89</v>
-      </c>
-      <c r="D26" t="n">
-        <v>313</v>
-      </c>
-      <c r="E26" t="n">
-        <v>243</v>
-      </c>
-      <c r="F26" t="n">
-        <v>30</v>
-      </c>
-      <c r="G26" t="n">
-        <v>7.38</v>
-      </c>
-      <c r="H26" t="n">
-        <v>1.86</v>
-      </c>
-      <c r="I26" t="n">
-        <v>11.18</v>
-      </c>
-      <c r="J26" t="n">
-        <v>17.52</v>
-      </c>
-      <c r="L26" t="n">
-        <v>3.64</v>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>PERFORMANCE GAP — shown, but CVR under target</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>B6</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Size: King</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>488.5000000000001</v>
-      </c>
-      <c r="D27" t="n">
-        <v>238</v>
-      </c>
-      <c r="E27" t="n">
-        <v>310</v>
-      </c>
-      <c r="F27" t="n">
-        <v>43</v>
-      </c>
-      <c r="G27" t="n">
-        <v>8.24</v>
-      </c>
-      <c r="H27" t="n">
-        <v>2.02</v>
-      </c>
-      <c r="I27" t="n">
-        <v>10.53</v>
-      </c>
-      <c r="J27" t="n">
-        <v>13.23</v>
-      </c>
-      <c r="L27" t="n">
-        <v>4.76</v>
-      </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>PERFORMANCE GAP — shown, but CVR under target</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>B6</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Size: Full</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>277.87</v>
-      </c>
-      <c r="D28" t="n">
-        <v>136</v>
-      </c>
-      <c r="E28" t="n">
-        <v>163</v>
-      </c>
-      <c r="F28" t="n">
-        <v>51</v>
-      </c>
-      <c r="G28" t="n">
-        <v>10.29</v>
-      </c>
-      <c r="H28" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="I28" t="n">
-        <v>6.68</v>
-      </c>
-      <c r="J28" t="n">
-        <v>18.9</v>
-      </c>
-      <c r="L28" t="n">
-        <v>4.28</v>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>PERFORMANCE GAP — shown, but CVR under target</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>B6</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Bamboo|Cooling</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>246.98</v>
-      </c>
-      <c r="D29" t="n">
-        <v>87</v>
-      </c>
-      <c r="E29" t="n">
-        <v>14</v>
-      </c>
-      <c r="F29" t="n">
-        <v>18</v>
-      </c>
-      <c r="G29" t="n">
-        <v>14.83</v>
-      </c>
-      <c r="H29" t="n">
-        <v>2.07</v>
-      </c>
-      <c r="I29" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="J29" t="n">
-        <v>7.71</v>
-      </c>
-      <c r="K29" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="L29" t="n">
-        <v>4.46</v>
-      </c>
-      <c r="M29" t="n">
-        <v>26</v>
-      </c>
-      <c r="N29" t="n">
-        <v>33</v>
-      </c>
-      <c r="O29" t="n">
-        <v>34</v>
-      </c>
-      <c r="P29" t="n">
-        <v>29</v>
-      </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>B6</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Bamboo|Twin</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>215.66</v>
-      </c>
-      <c r="D30" t="n">
-        <v>72</v>
-      </c>
-      <c r="E30" t="n">
-        <v>20</v>
-      </c>
-      <c r="F30" t="n">
-        <v>29</v>
-      </c>
-      <c r="G30" t="n">
-        <v>6.73</v>
-      </c>
-      <c r="H30" t="n">
-        <v>2.07</v>
-      </c>
-      <c r="I30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" t="n">
-        <v>10.95</v>
-      </c>
-      <c r="L30" t="n">
-        <v>5.34</v>
-      </c>
-      <c r="M30" t="n">
-        <v>7</v>
-      </c>
-      <c r="N30" t="n">
-        <v>15</v>
-      </c>
-      <c r="O30" t="n">
-        <v>20</v>
-      </c>
-      <c r="P30" t="n">
-        <v>20</v>
-      </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>PERFORMANCE GAP — shown, but CVR under target</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>B6</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Cooling|Queen</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>156.76</v>
-      </c>
-      <c r="D31" t="n">
-        <v>46</v>
-      </c>
-      <c r="E31" t="n">
-        <v>16</v>
-      </c>
-      <c r="F31" t="n">
-        <v>48</v>
-      </c>
-      <c r="G31" t="n">
-        <v>16.59</v>
-      </c>
-      <c r="H31" t="n">
-        <v>2.19</v>
-      </c>
-      <c r="I31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" t="n">
-        <v>12.3</v>
-      </c>
-      <c r="L31" t="n">
-        <v>4.59</v>
-      </c>
-      <c r="M31" t="n">
-        <v>38</v>
-      </c>
-      <c r="N31" t="n">
-        <v>67</v>
-      </c>
-      <c r="O31" t="n">
-        <v>81</v>
-      </c>
-      <c r="P31" t="n">
-        <v>75</v>
-      </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>B6</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Cooling|King</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>152.01</v>
-      </c>
-      <c r="D32" t="n">
-        <v>47</v>
-      </c>
-      <c r="E32" t="n">
-        <v>12</v>
-      </c>
-      <c r="F32" t="n">
-        <v>40</v>
-      </c>
-      <c r="G32" t="n">
-        <v>7.51</v>
-      </c>
-      <c r="H32" t="n">
-        <v>2.16</v>
-      </c>
-      <c r="I32" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="J32" t="n">
-        <v>10.53</v>
-      </c>
-      <c r="L32" t="n">
-        <v>5.54</v>
-      </c>
-      <c r="M32" t="n">
-        <v>48</v>
-      </c>
-      <c r="N32" t="n">
-        <v>59</v>
-      </c>
-      <c r="O32" t="n">
-        <v>43</v>
-      </c>
-      <c r="P32" t="n">
-        <v>40</v>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>TRAFFIC GAP — converts when shown, not shown/clicked enough</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>B6</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Bamboo|California King</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>107.54</v>
-      </c>
-      <c r="D33" t="n">
-        <v>39</v>
-      </c>
-      <c r="E33" t="n">
-        <v>2</v>
-      </c>
-      <c r="F33" t="n">
-        <v>5</v>
-      </c>
-      <c r="G33" t="n">
-        <v>6.66</v>
-      </c>
-      <c r="H33" t="n">
-        <v>2.07</v>
-      </c>
-      <c r="I33" t="n">
-        <v>0</v>
-      </c>
-      <c r="J33" t="n">
-        <v>8.85</v>
-      </c>
-      <c r="K33" t="n">
-        <v>2.01</v>
-      </c>
-      <c r="L33" t="n">
-        <v>3.24</v>
-      </c>
-      <c r="M33" t="n">
-        <v>26</v>
-      </c>
-      <c r="N33" t="n">
-        <v>16</v>
-      </c>
-      <c r="O33" t="n">
-        <v>34</v>
-      </c>
-      <c r="P33" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>B6</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Cooling|Full</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>86.13000000000001</v>
-      </c>
-      <c r="D34" t="n">
-        <v>22</v>
-      </c>
-      <c r="E34" t="n">
-        <v>16</v>
-      </c>
-      <c r="F34" t="n">
-        <v>73</v>
-      </c>
-      <c r="G34" t="n">
-        <v>10.27</v>
-      </c>
-      <c r="H34" t="n">
-        <v>2.18</v>
-      </c>
-      <c r="I34" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" t="n">
-        <v>12.42</v>
-      </c>
-      <c r="L34" t="n">
-        <v>4.64</v>
-      </c>
-      <c r="N34" t="n">
-        <v>56</v>
-      </c>
-      <c r="O34" t="n">
-        <v>87</v>
-      </c>
-      <c r="P34" t="n">
-        <v>87</v>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>BOTH — short of traffic and under target</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>B6</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Size: California King</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>65.81000000000002</v>
-      </c>
-      <c r="D35" t="n">
-        <v>30</v>
-      </c>
-      <c r="E35" t="n">
-        <v>12</v>
-      </c>
-      <c r="F35" t="n">
-        <v>17</v>
-      </c>
-      <c r="G35" t="n">
-        <v>21.69</v>
-      </c>
-      <c r="H35" t="n">
-        <v>1.94</v>
-      </c>
-      <c r="I35" t="n">
-        <v>6.12</v>
-      </c>
-      <c r="J35" t="n">
-        <v>15.78</v>
-      </c>
-      <c r="L35" t="n">
-        <v>2.98</v>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>B6</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Size: Twin</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>41.60999999999999</v>
-      </c>
-      <c r="D36" t="n">
-        <v>19</v>
-      </c>
-      <c r="E36" t="n">
-        <v>37</v>
-      </c>
-      <c r="F36" t="n">
-        <v>33</v>
-      </c>
-      <c r="G36" t="n">
-        <v>9.25</v>
-      </c>
-      <c r="H36" t="n">
-        <v>1.79</v>
-      </c>
-      <c r="I36" t="n">
-        <v>3.92</v>
-      </c>
-      <c r="J36" t="n">
-        <v>21.03</v>
-      </c>
-      <c r="L36" t="n">
-        <v>4.78</v>
-      </c>
-      <c r="Q36" t="inlineStr">
-        <is>
-          <t>PERFORMANCE GAP — shown, but CVR under target</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>B6</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Cooling|Twin</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>41.51</v>
-      </c>
-      <c r="D37" t="n">
-        <v>10</v>
-      </c>
-      <c r="E37" t="n">
-        <v>6</v>
-      </c>
-      <c r="F37" t="n">
-        <v>60</v>
-      </c>
-      <c r="G37" t="n">
-        <v>6.77</v>
-      </c>
-      <c r="H37" t="n">
-        <v>2.24</v>
-      </c>
-      <c r="I37" t="n">
-        <v>0</v>
-      </c>
-      <c r="J37" t="n">
-        <v>13.95</v>
-      </c>
-      <c r="L37" t="n">
-        <v>5.36</v>
-      </c>
-      <c r="M37" t="n">
-        <v>29</v>
-      </c>
-      <c r="N37" t="n">
-        <v>24</v>
-      </c>
-      <c r="O37" t="n">
-        <v>40</v>
-      </c>
-      <c r="P37" t="n">
-        <v>38</v>
-      </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>B6</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Cooling|California King</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>11.88</v>
-      </c>
-      <c r="D38" t="n">
-        <v>4</v>
-      </c>
-      <c r="E38" t="n">
-        <v>2</v>
-      </c>
-      <c r="F38" t="n">
-        <v>38</v>
-      </c>
-      <c r="G38" t="n">
-        <v>7.88</v>
-      </c>
-      <c r="H38" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="I38" t="n">
-        <v>0</v>
-      </c>
-      <c r="J38" t="n">
-        <v>10.05</v>
-      </c>
-      <c r="L38" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="M38" t="n">
-        <v>37</v>
-      </c>
-      <c r="N38" t="n">
-        <v>28</v>
-      </c>
-      <c r="O38" t="n">
-        <v>31</v>
-      </c>
-      <c r="P38" t="n">
-        <v>40</v>
-      </c>
-      <c r="Q38" t="inlineStr">
-        <is>
-          <t>NOT PRESENT at top of search</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Loss stop: use a campaign's own TOS conversion from 15 clicks (was 30)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FvXHKtbYmE3ru99HYV2muV
</commit_message>
<xml_diff>
--- a/docs/DBS4_Corrections_by_Situation_20260921-dbcd48b8.xlsx
+++ b/docs/DBS4_Corrections_by_Situation_20260921-dbcd48b8.xlsx
@@ -2468,7 +2468,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>Push TOS +20% (no click requirement on file → +20% (a stated departure: the logic document would hold at the ceiling)): $7.80 → $9.36; modifier 212%; daily read to 09-28</t>
+          <t>Push TOS +20% (loss stop reached — at 7.80 a top-of-search order already costs 94 (stop 3× contribution = 81)): $7.80 → $7.80; modifier 160%; daily read to 09-28</t>
         </is>
       </c>
     </row>
@@ -4606,7 +4606,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>Push TOS +30% (30% of required top-of-search clicks delivered → +30%; stopped at the loss stop 12.63): $9.76 → $12.63; modifier 430%; daily read to 09-28</t>
+          <t>Push TOS +30% (30% of required top-of-search clicks delivered → +30%): $9.76 → $12.69; modifier 433%; daily read to 09-28</t>
         </is>
       </c>
     </row>

</xml_diff>